<commit_message>
gestion des espaces dans le noms des lignes et colonnes
</commit_message>
<xml_diff>
--- a/New_Code/matrices.xlsx
+++ b/New_Code/matrices.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ipmc\Desktop\Code_hERG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guillaume\Desktop\hERG\New_Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BF471CC-3B10-4638-9F3B-D2B7A8F3F82C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12345" activeTab="2"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matrice des tailles" sheetId="1" r:id="rId1"/>
@@ -151,7 +152,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0_ ;\-0\ "/>
   </numFmts>
@@ -218,7 +219,7 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -233,7 +234,7 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -516,7 +517,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1888,7 +1889,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3260,23 +3261,23 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:21" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>4</v>
@@ -4434,7 +4435,7 @@
     </row>
     <row r="19" spans="1:21" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="B19" s="5">
         <v>0</v>

</xml_diff>

<commit_message>
moved variable choices from Chimer.py to main.py file
</commit_message>
<xml_diff>
--- a/New_Code/matrices.xlsx
+++ b/New_Code/matrices.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guillaume\Desktop\hERG\New_Code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ipmc\Desktop\Code_hERG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BF471CC-3B10-4638-9F3B-D2B7A8F3F82C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12345" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Matrice des tailles" sheetId="1" r:id="rId1"/>
@@ -152,7 +151,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0_ ;\-0\ "/>
   </numFmts>
@@ -219,7 +218,7 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -234,7 +233,7 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -517,7 +516,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1889,7 +1888,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3261,23 +3260,23 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:21" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>4</v>
@@ -4219,23 +4218,23 @@
       <c r="O15" s="4">
         <v>0</v>
       </c>
-      <c r="P15" s="6">
-        <v>1</v>
+      <c r="P15" s="7">
+        <v>2</v>
       </c>
       <c r="Q15" s="6">
         <v>1</v>
       </c>
-      <c r="R15" s="6">
-        <v>1</v>
+      <c r="R15" s="7">
+        <v>2</v>
       </c>
       <c r="S15" s="6">
         <v>1</v>
       </c>
-      <c r="T15" s="6">
-        <v>1</v>
-      </c>
-      <c r="U15" s="6">
-        <v>1</v>
+      <c r="T15" s="5">
+        <v>0</v>
+      </c>
+      <c r="U15" s="5">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="18.75" x14ac:dyDescent="0.25">
@@ -4281,8 +4280,8 @@
       <c r="N16" s="6">
         <v>1</v>
       </c>
-      <c r="O16" s="6">
-        <v>1</v>
+      <c r="O16" s="7">
+        <v>2</v>
       </c>
       <c r="P16" s="4">
         <v>0</v>
@@ -4411,8 +4410,8 @@
       <c r="N18" s="6">
         <v>1</v>
       </c>
-      <c r="O18" s="6">
-        <v>1</v>
+      <c r="O18" s="7">
+        <v>2</v>
       </c>
       <c r="P18" s="5">
         <v>0</v>
@@ -4435,7 +4434,7 @@
     </row>
     <row r="19" spans="1:21" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B19" s="5">
         <v>0</v>
@@ -4541,8 +4540,8 @@
       <c r="N20" s="6">
         <v>1</v>
       </c>
-      <c r="O20" s="6">
-        <v>1</v>
+      <c r="O20" s="5">
+        <v>0</v>
       </c>
       <c r="P20" s="7">
         <v>2</v>
@@ -4606,8 +4605,8 @@
       <c r="N21" s="6">
         <v>1</v>
       </c>
-      <c r="O21" s="6">
-        <v>1</v>
+      <c r="O21" s="5">
+        <v>0</v>
       </c>
       <c r="P21" s="7">
         <v>2</v>

</xml_diff>